<commit_message>
Included screenshots in extent report
</commit_message>
<xml_diff>
--- a/BrowserStackEcommerce_Automation/src/main/java/com/bstack/testdata/LoginData.xlsx
+++ b/BrowserStackEcommerce_Automation/src/main/java/com/bstack/testdata/LoginData.xlsx
@@ -27,16 +27,16 @@
     <t>Password</t>
   </si>
   <si>
-    <t>Lakshmisri</t>
-  </si>
-  <si>
-    <t>akanksha@123</t>
-  </si>
-  <si>
     <t>demouser</t>
   </si>
   <si>
     <t>testingisfun99</t>
+  </si>
+  <si>
+    <t>testing99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
@@ -382,26 +382,26 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -412,8 +412,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" display="lakshmisri@123"/>
-    <hyperlink ref="B4" r:id="rId2"/>
+    <hyperlink ref="B4" r:id="rId1" display="lakshmisri@123"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added browser name in screensot name and included screenshots in extent report
</commit_message>
<xml_diff>
--- a/BrowserStackEcommerce_Automation/src/main/java/com/bstack/testdata/LoginData.xlsx
+++ b/BrowserStackEcommerce_Automation/src/main/java/com/bstack/testdata/LoginData.xlsx
@@ -43,7 +43,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -59,13 +59,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -81,9 +95,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -365,7 +380,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" customWidth="1"/>
@@ -373,10 +388,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -403,17 +418,12 @@
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B5" s="1"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B6" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" display="lakshmisri@123"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>